<commit_message>
Tighten news filtering, clean titles, chip nowrap
</commit_message>
<xml_diff>
--- a/data/source/AMR_Master_20261021.xlsx
+++ b/data/source/AMR_Master_20261021.xlsx
@@ -14262,7 +14262,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>salmon, kingfish, barramundi, bluefin tuna ranching, sea cage, fish farm, tassal, huon aquaculture, petuna, macquarie harbour</t>
+          <t>salmon farm, salmon farming, salmon industry, salmon producer, kingfish, barramundi farm, bluefin tuna ranching, tuna farm, sea cage, fish farm, tassal, huon aquaculture, petuna, macquarie harbour</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -14284,7 +14284,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>oyster, mussel, abalone farm, pearl, paspaley</t>
+          <t>oyster farm, oyster industry, oysters, oyster lease, mussel farm, abalone farm, pearl farm, pearling, paspaley</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>fishery, fisheries, rock lobster, prawn, afma, quota, total allowable catch, trawl, gillnet, toothfish</t>
+          <t>fishery, fisheries, rock lobster, prawn fishery, prawn trawl, prawn catch, afma, total allowable catch, fishing quota, commercial fishing, trawler, gillnet, toothfish</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">

</xml_diff>